<commit_message>
Add canonical facade regression workflow and socle fixes
</commit_message>
<xml_diff>
--- a/assets/test_output.xlsx
+++ b/assets/test_output.xlsx
@@ -562,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -570,8 +570,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generat: 03.03.2026 10:55</t>
+          <t>Generat: 05.03.2026 17:47</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>F_3</t>
+          <t>F_6</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -671,95 +671,95 @@
       <c r="E6" s="8" t="inlineStr"/>
       <c r="F6" s="8" t="inlineStr"/>
       <c r="G6" s="9" t="n">
-        <v>0</v>
+        <v>1.091</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr"/>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>FATADA PRINCIPALA</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>F_3</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Fereastra</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr"/>
+      <c r="G7" s="9" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>FATADA PRINCIPALA</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>U2</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Usa</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr"/>
-      <c r="F7" s="11" t="inlineStr"/>
-      <c r="G7" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="12" t="n">
+        <v>1.005</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  Subtotal FATADA PRINCIPALA</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="15" t="n">
-        <v>24.29</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="B9" s="14" t="n"/>
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="15" t="n">
+        <v>3.866</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>20.424</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>FATADA LATERALA STANGA</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>FATADA</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Termosistem</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr"/>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>FATADA LATERALA STANGA</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Fereastra</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
-      <c r="G10" s="9" t="n">
-        <v>2.28</v>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="6" t="n">
+        <v>71.039</v>
       </c>
     </row>
     <row r="11">
@@ -782,30 +782,30 @@
       <c r="E11" s="8" t="inlineStr"/>
       <c r="F11" s="8" t="inlineStr"/>
       <c r="G11" s="9" t="n">
+        <v>2.28</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>FATADA LATERALA STANGA</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Fereastra</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr"/>
+      <c r="G12" s="9" t="n">
         <v>2.26</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>FATADA LATERALA STANGA</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>U_6</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>Usa</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr"/>
-      <c r="F12" s="11" t="inlineStr"/>
-      <c r="G12" s="12" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -822,7 +822,7 @@
         <v>4.539999999999999</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>0</v>
+        <v>66.499</v>
       </c>
     </row>
     <row r="14">
@@ -870,142 +870,126 @@
       <c r="E15" s="8" t="inlineStr"/>
       <c r="F15" s="8" t="inlineStr"/>
       <c r="G15" s="9" t="n">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>FATADA POSTERIOARA</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>F_2</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Fereastra</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr"/>
+      <c r="G16" s="9" t="n">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Subtotal FATADA POSTERIOARA</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n"/>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="15" t="n">
+        <v>4.539999999999999</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>54.32</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>FATADA LATERALA DREAPTA</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>FATADA</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Termosistem</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="6" t="n">
+        <v>31.53</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Subtotal FATADA LATERALA DREAPTA</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="15" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr"/>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>FATADA POSTERIOARA</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>U_3</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>Usa</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr"/>
-      <c r="F16" s="11" t="inlineStr"/>
-      <c r="G16" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr"/>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>FATADA POSTERIOARA</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>U_1</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Usa</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="inlineStr"/>
-      <c r="F17" s="11" t="inlineStr"/>
-      <c r="G17" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Subtotal FATADA POSTERIOARA</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
-      <c r="F18" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="15" t="n">
-        <v>58.86</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>FATADA LATERALA DREAPTA</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>FATADA</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Termosistem</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr"/>
-      <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="15" t="n">
         <v>31.53</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr"/>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>FATADA LATERALA DREAPTA</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>U_2</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Usa</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr"/>
-      <c r="F20" s="11" t="inlineStr"/>
-      <c r="G20" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Subtotal FATADA LATERALA DREAPTA</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="15" t="n">
-        <v>31.53</v>
-      </c>
-    </row>
-    <row r="22"/>
+    <row r="20"/>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL SUPRAFATA FATADE</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="17" t="n"/>
+      <c r="G21" s="18" t="n">
+        <v>185.719</v>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL TAMPLARIE (Ferestre + Usi)</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="18" t="n">
+        <v>12.946</v>
+      </c>
+    </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>TOTAL SUPRAFATA FATADE</t>
+          <t>TOTAL TERMOSISTEM (Fatade - Tamplarie)</t>
         </is>
       </c>
       <c r="B23" s="17" t="n"/>
@@ -1014,13 +998,13 @@
       <c r="E23" s="17" t="n"/>
       <c r="F23" s="17" t="n"/>
       <c r="G23" s="18" t="n">
-        <v>114.68</v>
+        <v>172.773</v>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>TOTAL TAMPLARIE (Ferestre + Usi)</t>
+          <t>TOTAL SOCLU EXCLUS</t>
         </is>
       </c>
       <c r="B24" s="17" t="n"/>
@@ -1029,13 +1013,13 @@
       <c r="E24" s="17" t="n"/>
       <c r="F24" s="17" t="n"/>
       <c r="G24" s="18" t="n">
-        <v>4.539999999999999</v>
+        <v>10.705</v>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>TOTAL TERMOSISTEM (Fatade - Tamplarie)</t>
+          <t>TOTAL LUNGIME GLAF</t>
         </is>
       </c>
       <c r="B25" s="17" t="n"/>
@@ -1044,19 +1028,53 @@
       <c r="E25" s="17" t="n"/>
       <c r="F25" s="17" t="n"/>
       <c r="G25" s="18" t="n">
-        <v>114.68</v>
+        <v>6.594</v>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL LUNGIME PICURATOR</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="17" t="n"/>
+      <c r="D26" s="17" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="18" t="n">
+        <v>7.962</v>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL LUNGIME COLTARE</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="n"/>
+      <c r="C27" s="17" t="n"/>
+      <c r="D27" s="17" t="n"/>
+      <c r="E27" s="17" t="n"/>
+      <c r="F27" s="17" t="n"/>
+      <c r="G27" s="18" t="n">
+        <v>61.65</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A21:E21"/>
+  <mergeCells count="13">
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1069,13 +1087,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1106,6 +1128,26 @@
           <t>Termosistem (m²)</t>
         </is>
       </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Soclu exclus (m²)</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>Glaf (m)</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Picurator (m)</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>Coltare (m)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
@@ -1117,10 +1159,22 @@
         <v>24.29</v>
       </c>
       <c r="C4" s="22" t="n">
+        <v>3.866</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <v>20.424</v>
+      </c>
+      <c r="E4" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="22" t="n">
-        <v>24.29</v>
+      <c r="F4" s="22" t="n">
+        <v>2.165</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>3.533</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>16.271</v>
       </c>
     </row>
     <row r="5">
@@ -1130,13 +1184,25 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0</v>
+        <v>71.039</v>
       </c>
       <c r="C5" s="22" t="n">
         <v>4.539999999999999</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>0</v>
+        <v>66.499</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>10.705</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>2.289</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>2.289</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>12.539</v>
       </c>
     </row>
     <row r="6">
@@ -1149,10 +1215,22 @@
         <v>58.86</v>
       </c>
       <c r="C6" s="22" t="n">
+        <v>4.539999999999999</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>54.32</v>
+      </c>
+      <c r="E6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="22" t="n">
-        <v>58.86</v>
+      <c r="F6" s="22" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="G6" s="22" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>13.136</v>
       </c>
     </row>
     <row r="7">
@@ -1170,6 +1248,18 @@
       <c r="D7" s="22" t="n">
         <v>31.53</v>
       </c>
+      <c r="E7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <v>19.704</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
@@ -1178,18 +1268,30 @@
         </is>
       </c>
       <c r="B8" s="24" t="n">
-        <v>114.68</v>
+        <v>185.719</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>4.539999999999999</v>
+        <v>12.946</v>
       </c>
       <c r="D8" s="24" t="n">
-        <v>114.68</v>
+        <v>172.773</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>10.705</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>6.594</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>7.962</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>61.65</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>